<commit_message>
added the latest GPU benchmarks results to excel files and python scripts
</commit_message>
<xml_diff>
--- a/benchmarks_tests/FINAL_Benchmarks_for_paper/PyFock_CPU_vs_GPU.xlsx
+++ b/benchmarks_tests/FINAL_Benchmarks_for_paper/PyFock_CPU_vs_GPU.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/manas/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/manas/Documents/PyFock/benchmarks_tests/FINAL_Benchmarks_for_paper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7668C041-413D-7741-A016-199E21B6398F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFAD117A-340D-F943-B3BB-008BD4E89C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1080" yWindow="1260" windowWidth="27640" windowHeight="16460" xr2:uid="{0352C87C-B4A4-4D4C-883B-F1396BEEBBFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="26">
   <si>
     <t>PyFock CPU vs GPU</t>
   </si>
@@ -99,6 +99,21 @@
   </si>
   <si>
     <t>J  / iter (s) (GPU)</t>
+  </si>
+  <si>
+    <t>Cholesky off</t>
+  </si>
+  <si>
+    <t>save ao off</t>
+  </si>
+  <si>
+    <t>xc block 20480</t>
+  </si>
+  <si>
+    <t>3c2e ints threads 8x8</t>
+  </si>
+  <si>
+    <t>max register 800</t>
   </si>
 </sst>
 </file>
@@ -522,16 +537,31 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
@@ -572,20 +602,18 @@
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
-      <c r="F6" s="2">
-        <v>8</v>
-      </c>
-      <c r="G6">
+      <c r="F6" s="2"/>
+      <c r="G6" t="e">
         <f>C6/F6</f>
-        <v>0</v>
-      </c>
-      <c r="H6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H6" t="e">
         <f>D6/F6</f>
-        <v>0</v>
-      </c>
-      <c r="I6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I6" t="e">
         <f>E6/F6</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
@@ -595,29 +623,21 @@
       <c r="B7">
         <v>125</v>
       </c>
-      <c r="C7" s="2">
-        <v>2.9560983460396502</v>
-      </c>
-      <c r="D7" s="2">
-        <v>0.42427957803010902</v>
-      </c>
-      <c r="E7" s="2">
-        <v>0.86814015824347701</v>
-      </c>
-      <c r="F7" s="2">
-        <v>10</v>
-      </c>
-      <c r="G7">
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" t="e">
         <f t="shared" ref="G7:G14" si="0">C7/F7</f>
-        <v>0.295609834603965</v>
-      </c>
-      <c r="H7">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H7" t="e">
         <f t="shared" ref="H7:H14" si="1">D7/F7</f>
-        <v>4.2427957803010903E-2</v>
-      </c>
-      <c r="I7">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I7" t="e">
         <f t="shared" ref="I7:I14" si="2">E7/F7</f>
-        <v>8.6814015824347696E-2</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
@@ -660,28 +680,28 @@
         <v>500</v>
       </c>
       <c r="C9" s="2">
-        <v>6.0103211449459097</v>
+        <v>5.7691683680750403</v>
       </c>
       <c r="D9" s="2">
-        <v>2.4581313524395201</v>
+        <v>2.1158297739457299</v>
       </c>
       <c r="E9" s="2">
-        <v>1.7156712030991901</v>
+        <v>2.0066158876288598</v>
       </c>
       <c r="F9" s="2">
         <v>13</v>
       </c>
       <c r="G9">
         <f t="shared" si="0"/>
-        <v>0.46233239576506996</v>
+        <v>0.44378218215961851</v>
       </c>
       <c r="H9">
         <f t="shared" si="1"/>
-        <v>0.1890870271107323</v>
+        <v>0.16275613645736384</v>
       </c>
       <c r="I9">
         <f t="shared" si="2"/>
-        <v>0.13197470793070692</v>
+        <v>0.15435506827914305</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -692,28 +712,28 @@
         <v>800</v>
       </c>
       <c r="C10" s="2">
-        <v>13.9464681548997</v>
+        <v>12.2090913550928</v>
       </c>
       <c r="D10" s="2">
-        <v>6.0748179610818598</v>
+        <v>5.2523773421998996</v>
       </c>
       <c r="E10" s="2">
-        <v>4.0294136004522398</v>
+        <v>3.9277749070897698</v>
       </c>
       <c r="F10" s="2">
         <v>15</v>
       </c>
       <c r="G10">
         <f t="shared" si="0"/>
-        <v>0.92976454365997996</v>
+        <v>0.81393942367285332</v>
       </c>
       <c r="H10">
         <f t="shared" si="1"/>
-        <v>0.404987864072124</v>
+        <v>0.35015848947999328</v>
       </c>
       <c r="I10">
         <f t="shared" si="2"/>
-        <v>0.26862757336348264</v>
+        <v>0.26185166047265135</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
@@ -724,28 +744,28 @@
         <v>1175</v>
       </c>
       <c r="C11" s="2">
-        <v>27.236856956034899</v>
+        <v>23.0492668540682</v>
       </c>
       <c r="D11" s="2">
-        <v>13.445535489358001</v>
+        <v>11.764931902987801</v>
       </c>
       <c r="E11" s="2">
-        <v>7.2065506465732998</v>
+        <v>6.2060886947438103</v>
       </c>
       <c r="F11" s="2">
         <v>15</v>
       </c>
       <c r="G11">
         <f t="shared" si="0"/>
-        <v>1.8157904637356599</v>
+        <v>1.5366177902712133</v>
       </c>
       <c r="H11">
         <f t="shared" si="1"/>
-        <v>0.89636903262386669</v>
+        <v>0.78432879353252005</v>
       </c>
       <c r="I11">
         <f t="shared" si="2"/>
-        <v>0.48043670977155334</v>
+        <v>0.41373924631625403</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
@@ -756,28 +776,28 @@
         <v>1900</v>
       </c>
       <c r="C12" s="2">
-        <v>69.871257518418105</v>
+        <v>55.972384363878497</v>
       </c>
       <c r="D12" s="2">
-        <v>36.925900157541001</v>
+        <v>31.8730793460272</v>
       </c>
       <c r="E12" s="2">
-        <v>16.8591308072209</v>
+        <v>13.263924242928599</v>
       </c>
       <c r="F12" s="2">
         <v>17</v>
       </c>
       <c r="G12">
         <f t="shared" si="0"/>
-        <v>4.1100739716716532</v>
+        <v>3.2924931978752059</v>
       </c>
       <c r="H12">
         <f t="shared" si="1"/>
-        <v>2.172111773973</v>
+        <v>1.8748870203545411</v>
       </c>
       <c r="I12">
         <f t="shared" si="2"/>
-        <v>0.99171357689534712</v>
+        <v>0.78023083781932934</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -788,28 +808,28 @@
         <v>2500</v>
       </c>
       <c r="C13" s="2">
-        <v>114.97582897730101</v>
+        <v>88.581307347165406</v>
       </c>
       <c r="D13" s="2">
-        <v>67.9061539517715</v>
+        <v>57.356785830110297</v>
       </c>
       <c r="E13" s="2">
-        <v>20.950647555291599</v>
+        <v>16.1813672701828</v>
       </c>
       <c r="F13" s="2">
         <v>15</v>
       </c>
       <c r="G13">
         <f t="shared" si="0"/>
-        <v>7.6650552651534003</v>
+        <v>5.9054204898110267</v>
       </c>
       <c r="H13">
         <f t="shared" si="1"/>
-        <v>4.5270769301181</v>
+        <v>3.823785722007353</v>
       </c>
       <c r="I13">
         <f t="shared" si="2"/>
-        <v>1.39670983701944</v>
+        <v>1.0787578180121866</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
@@ -820,28 +840,28 @@
         <v>3475</v>
       </c>
       <c r="C14" s="2">
-        <v>231.74738594610201</v>
+        <v>171.51697664405199</v>
       </c>
       <c r="D14" s="2">
-        <v>136.71365584619301</v>
+        <v>114.241373233031</v>
       </c>
       <c r="E14" s="2">
-        <v>35.890776604413901</v>
+        <v>26.2381101583596</v>
       </c>
       <c r="F14" s="2">
         <v>16</v>
       </c>
       <c r="G14">
         <f t="shared" si="0"/>
-        <v>14.484211621631376</v>
+        <v>10.71981104025325</v>
       </c>
       <c r="H14">
         <f t="shared" si="1"/>
-        <v>8.5446034903870629</v>
+        <v>7.1400858270644374</v>
       </c>
       <c r="I14">
         <f t="shared" si="2"/>
-        <v>2.2431735377758688</v>
+        <v>1.639881884897475</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
@@ -1177,20 +1197,11 @@
       <c r="B34" s="3">
         <v>125</v>
       </c>
-      <c r="C34">
-        <v>0.295609834603965</v>
-      </c>
       <c r="D34">
         <v>0.25187982799999997</v>
       </c>
-      <c r="E34">
-        <v>4.2427957803010903E-2</v>
-      </c>
       <c r="F34">
         <v>8.2255138000000005E-2</v>
-      </c>
-      <c r="G34">
-        <v>8.6814015824347696E-2</v>
       </c>
       <c r="H34">
         <v>0.10870471</v>
@@ -1230,19 +1241,19 @@
         <v>500</v>
       </c>
       <c r="C36">
-        <v>0.46233239576506996</v>
+        <v>0.44378218215961851</v>
       </c>
       <c r="D36">
         <v>3.3269480499999999</v>
       </c>
       <c r="E36">
-        <v>0.1890870271107323</v>
+        <v>0.16275613645736384</v>
       </c>
       <c r="F36">
         <v>1.910627895</v>
       </c>
       <c r="G36">
-        <v>0.13197470793070692</v>
+        <v>0.15435506827914305</v>
       </c>
       <c r="H36">
         <v>0.95263880999999995</v>
@@ -1256,19 +1267,19 @@
         <v>800</v>
       </c>
       <c r="C37">
-        <v>0.92976454365997996</v>
+        <v>0.81393942367285332</v>
       </c>
       <c r="D37">
         <v>7.5122146250000004</v>
       </c>
       <c r="E37">
-        <v>0.404987864072124</v>
+        <v>0.35015848947999328</v>
       </c>
       <c r="F37">
         <v>4.4082032179999997</v>
       </c>
       <c r="G37">
-        <v>0.26862757336348264</v>
+        <v>0.26185166047265135</v>
       </c>
       <c r="H37">
         <v>1.9939018500000001</v>
@@ -1282,19 +1293,19 @@
         <v>1175</v>
       </c>
       <c r="C38">
-        <v>1.8157904637356599</v>
+        <v>1.5366177902712133</v>
       </c>
       <c r="D38">
         <v>17.15226698</v>
       </c>
       <c r="E38">
-        <v>0.89636903262386669</v>
+        <v>0.78432879353252005</v>
       </c>
       <c r="F38">
         <v>10.75980461</v>
       </c>
       <c r="G38">
-        <v>0.48043670977155334</v>
+        <v>0.41373924631625403</v>
       </c>
       <c r="H38">
         <v>3.7608596699999999</v>
@@ -1308,19 +1319,19 @@
         <v>1900</v>
       </c>
       <c r="C39">
-        <v>4.1100739716716532</v>
+        <v>3.2924931978752059</v>
       </c>
       <c r="D39">
         <v>41.328410030000001</v>
       </c>
       <c r="E39">
-        <v>2.172111773973</v>
+        <v>1.8748870203545411</v>
       </c>
       <c r="F39">
         <v>24.763817299999999</v>
       </c>
       <c r="G39">
-        <v>0.99171357689534712</v>
+        <v>0.78023083781932934</v>
       </c>
       <c r="H39">
         <v>8.6174155700000004</v>
@@ -1334,19 +1345,19 @@
         <v>2500</v>
       </c>
       <c r="C40">
-        <v>7.6650552651534003</v>
+        <v>5.9054204898110267</v>
       </c>
       <c r="D40">
         <v>82.384753419999996</v>
       </c>
       <c r="E40">
-        <v>4.5270769301181</v>
+        <v>3.823785722007353</v>
       </c>
       <c r="F40">
         <v>54.06537282</v>
       </c>
       <c r="G40">
-        <v>1.39670983701944</v>
+        <v>1.0787578180121866</v>
       </c>
       <c r="H40">
         <v>12.6850703</v>
@@ -1360,19 +1371,19 @@
         <v>3475</v>
       </c>
       <c r="C41">
-        <v>14.484211621631376</v>
+        <v>10.71981104025325</v>
       </c>
       <c r="D41">
         <v>154.2059581</v>
       </c>
       <c r="E41">
-        <v>8.5446034903870629</v>
+        <v>7.1400858270644374</v>
       </c>
       <c r="F41">
         <v>97.104628309999995</v>
       </c>
       <c r="G41">
-        <v>2.2431735377758688</v>
+        <v>1.639881884897475</v>
       </c>
       <c r="H41">
         <v>21.373439000000001</v>

</xml_diff>